<commit_message>
Piani e prova gratuita: listino v3, limiti, estensioni, landing, account di prova
</commit_message>
<xml_diff>
--- a/Fatture/Registro-Spese.xlsx
+++ b/Fatture/Registro-Spese.xlsx
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-08 09:30:52</t>
+          <t>2026-10-06 11:47:08</t>
         </is>
       </c>
     </row>
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>57.17</v>
+        <v>81.72</v>
       </c>
     </row>
     <row r="7">
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>10.31</v>
+        <v>14.74</v>
       </c>
     </row>
     <row r="8">
@@ -559,7 +559,7 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>250.1</v>
+        <v>265.96</v>
       </c>
     </row>
     <row r="14">
@@ -570,7 +570,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-10-13 — IONOS VPS Linux L+ (trainmind-vps) (35 gg)</t>
+          <t>2026-10-13 — IONOS VPS Linux L+ (trainmind-vps) (7 gg)</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1098,6 +1098,75 @@
       </c>
       <c r="Q7" t="inlineStr"/>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>IONOS SE</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Infrastruttura</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>IONOS VPS Linux L+</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>109994221094</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>20.12</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>24.55</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>20.12</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>24.55</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>ionos/Fattura_2026-09-16_109994221094_V112969652.pdf</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1179,13 +1248,13 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>6.5</v>
+        <v>26.62</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1.43</v>
+        <v>5.86</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>7.93</v>
+        <v>32.48</v>
       </c>
     </row>
   </sheetData>
@@ -1478,11 +1547,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1511,7 +1580,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>308</v>
+        <v>280</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -1570,7 +1639,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="B2" s="4" t="n">
@@ -1580,17 +1649,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>2026-11</t>
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>6.1</v>
+        <v>21.96</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-11</t>
+          <t>2026-12</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
@@ -1600,7 +1669,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-12</t>
+          <t>2027-01</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
@@ -1610,7 +1679,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2027-01</t>
+          <t>2027-02</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
@@ -1620,7 +1689,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2027-02</t>
+          <t>2027-03</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
@@ -1630,7 +1699,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2027-03</t>
+          <t>2027-04</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
@@ -1640,7 +1709,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2027-04</t>
+          <t>2027-05</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
@@ -1650,7 +1719,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2027-05</t>
+          <t>2027-06</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
@@ -1660,27 +1729,27 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2027-06</t>
+          <t>2027-07</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>21.96</v>
+        <v>40.26</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2027-07</t>
+          <t>2027-08</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>40.26</v>
+        <v>21.96</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2027-08</t>
+          <t>2027-09</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
@@ -1694,7 +1763,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>250.1</v>
+        <v>265.96</v>
       </c>
     </row>
   </sheetData>
@@ -1734,7 +1803,7 @@
         </is>
       </c>
       <c r="B2" s="4" t="n">
-        <v>10.31</v>
+        <v>14.74</v>
       </c>
     </row>
     <row r="3">
@@ -1744,7 +1813,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>10.31</v>
+        <v>14.74</v>
       </c>
     </row>
   </sheetData>
@@ -1832,7 +1901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2377,6 +2446,192 @@
         <v>22</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>IONOS SE</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>109994221094</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Tariﬀa base</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="G18" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>IONOS SE</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>109994221094</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Sconto</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>-13</v>
+      </c>
+      <c r="G19" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>IONOS SE</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>109994221094</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>IP addizionale</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>IONOS SE</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>109994221094</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>4</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>IONOS Cloud</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>14.52</v>
+      </c>
+      <c r="G21" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>IONOS SE</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>109994221094</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>5</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>IONOS Cloud</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G22" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>IONOS SE</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>109994221094</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>6</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>IP addizionale</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>